<commit_message>
#62 Updated Files Client BOM for Hub Design
</commit_message>
<xml_diff>
--- a/Deliverables/HUB/BOM/Client_BOM_Ezlo_Voice_AssistantHUB.xlsx
+++ b/Deliverables/HUB/BOM/Client_BOM_Ezlo_Voice_AssistantHUB.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Ezlo-VoiceAssistant\Deliverables\HUB\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4C9F151-1C91-4840-BA60-583F120B86A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6157CD6-E7D3-4CBC-970A-A2E6EE27ED91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="515">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1014" uniqueCount="515">
   <si>
     <t>Component list</t>
   </si>
@@ -2202,6 +2202,15 @@
     <xf numFmtId="165" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="23" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2218,15 +2227,6 @@
     <xf numFmtId="0" fontId="21" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="23" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2600,13 +2600,13 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="70"/>
-      <c r="K1" s="70"/>
-      <c r="L1" s="70"/>
-      <c r="M1" s="70"/>
-      <c r="N1" s="70"/>
-      <c r="O1" s="70"/>
-      <c r="P1" s="70"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
+      <c r="L1" s="73"/>
+      <c r="M1" s="73"/>
+      <c r="N1" s="73"/>
+      <c r="O1" s="73"/>
+      <c r="P1" s="73"/>
     </row>
     <row r="2" spans="1:16" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2650,7 +2650,7 @@
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
-      <c r="P3" s="71"/>
+      <c r="P3" s="74"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -2672,7 +2672,7 @@
       <c r="M4" s="5"/>
       <c r="N4" s="5"/>
       <c r="O4" s="5"/>
-      <c r="P4" s="72"/>
+      <c r="P4" s="75"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -2694,7 +2694,7 @@
       <c r="M5" s="5"/>
       <c r="N5" s="5"/>
       <c r="O5" s="5"/>
-      <c r="P5" s="72"/>
+      <c r="P5" s="75"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -2712,7 +2712,7 @@
       <c r="M6" s="5"/>
       <c r="N6" s="5"/>
       <c r="O6" s="5"/>
-      <c r="P6" s="72"/>
+      <c r="P6" s="75"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2730,7 +2730,7 @@
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
       <c r="O7" s="7"/>
-      <c r="P7" s="72"/>
+      <c r="P7" s="75"/>
     </row>
     <row r="8" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2748,7 +2748,7 @@
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>
       <c r="O8" s="7"/>
-      <c r="P8" s="72"/>
+      <c r="P8" s="75"/>
     </row>
     <row r="9" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -7174,26 +7174,28 @@
       <c r="D101" s="38" t="s">
         <v>97</v>
       </c>
-      <c r="E101" s="75" t="s">
+      <c r="E101" s="70" t="s">
         <v>208</v>
       </c>
-      <c r="F101" s="76" t="s">
+      <c r="F101" s="71" t="s">
         <v>487</v>
       </c>
-      <c r="G101" s="75" t="s">
+      <c r="G101" s="70" t="s">
         <v>266</v>
       </c>
-      <c r="H101" s="76"/>
-      <c r="I101" s="76" t="s">
+      <c r="H101" s="71" t="s">
+        <v>480</v>
+      </c>
+      <c r="I101" s="71" t="s">
         <v>393</v>
       </c>
-      <c r="J101" s="76" t="s">
-        <v>480</v>
-      </c>
-      <c r="K101" s="75">
+      <c r="J101" s="71" t="s">
+        <v>480</v>
+      </c>
+      <c r="K101" s="70">
         <v>1</v>
       </c>
-      <c r="L101" s="76">
+      <c r="L101" s="71">
         <v>11</v>
       </c>
       <c r="M101" s="64" t="s">
@@ -7202,7 +7204,7 @@
       <c r="N101" s="65">
         <v>0.3</v>
       </c>
-      <c r="O101" s="77">
+      <c r="O101" s="72">
         <f t="shared" si="2"/>
         <v>3.3</v>
       </c>
@@ -8084,11 +8086,11 @@
       <c r="I120" s="34"/>
       <c r="J120" s="35"/>
       <c r="K120" s="35"/>
-      <c r="L120" s="73" t="s">
+      <c r="L120" s="76" t="s">
         <v>510</v>
       </c>
-      <c r="M120" s="74"/>
-      <c r="N120" s="74"/>
+      <c r="M120" s="77"/>
+      <c r="N120" s="77"/>
       <c r="O120" s="66">
         <f>SUM(O10:O119)</f>
         <v>1787.6428999999998</v>
@@ -8107,11 +8109,11 @@
       <c r="I121" s="9"/>
       <c r="J121" s="9"/>
       <c r="K121" s="9"/>
-      <c r="L121" s="73" t="s">
+      <c r="L121" s="76" t="s">
         <v>511</v>
       </c>
-      <c r="M121" s="74"/>
-      <c r="N121" s="74"/>
+      <c r="M121" s="77"/>
+      <c r="N121" s="77"/>
       <c r="O121" s="67">
         <f>O120/10</f>
         <v>178.76428999999999</v>

</xml_diff>

<commit_message>
#56 Updated Hub Client BOM and eSpark BOM.
</commit_message>
<xml_diff>
--- a/Deliverables/HUB/BOM/Client_BOM_Ezlo_Voice_AssistantHUB.xlsx
+++ b/Deliverables/HUB/BOM/Client_BOM_Ezlo_Voice_AssistantHUB.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Ezlo-VoiceAssistant\Deliverables\HUB\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6157CD6-E7D3-4CBC-970A-A2E6EE27ED91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F702FE6E-EABA-41AB-8B1E-62B414FBE125}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1014" uniqueCount="515">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="905" uniqueCount="514">
   <si>
     <t>Component list</t>
   </si>
@@ -1550,9 +1550,6 @@
     <t>0603WAJ0220T5E</t>
   </si>
   <si>
-    <t>Links</t>
-  </si>
-  <si>
     <t>Unit Cost (10 Boards)</t>
   </si>
   <si>
@@ -1574,7 +1571,7 @@
     <t>[HUB_Design]</t>
   </si>
   <si>
-    <t>Self Supplier</t>
+    <t>Quantity (10 Boards)</t>
   </si>
 </sst>
 </file>
@@ -1586,7 +1583,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1720,14 +1717,6 @@
       <strike/>
       <sz val="9"/>
       <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2008,11 +1997,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2178,13 +2166,7 @@
     <xf numFmtId="0" fontId="19" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="165" fontId="17" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="17" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2196,19 +2178,19 @@
     <xf numFmtId="166" fontId="14" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="23" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="22" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2220,17 +2202,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2583,8 +2564,8 @@
     <col min="9" max="9" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="7.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="19.7109375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="20.28515625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="29.42578125" customWidth="1"/>
@@ -2600,13 +2581,13 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="73"/>
-      <c r="K1" s="73"/>
-      <c r="L1" s="73"/>
-      <c r="M1" s="73"/>
-      <c r="N1" s="73"/>
-      <c r="O1" s="73"/>
-      <c r="P1" s="73"/>
+      <c r="J1" s="71"/>
+      <c r="K1" s="71"/>
+      <c r="L1" s="71"/>
+      <c r="M1" s="71"/>
+      <c r="N1" s="71"/>
+      <c r="O1" s="71"/>
+      <c r="P1" s="71"/>
     </row>
     <row r="2" spans="1:16" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2617,7 +2598,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="52" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
@@ -2639,7 +2620,7 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="53" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
@@ -2650,7 +2631,7 @@
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
-      <c r="P3" s="74"/>
+      <c r="P3" s="72"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -2661,18 +2642,18 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="54" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
       <c r="I4" s="6"/>
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="5"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="6"/>
       <c r="N4" s="5"/>
       <c r="O4" s="5"/>
-      <c r="P4" s="75"/>
+      <c r="P4" s="73"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -2694,7 +2675,7 @@
       <c r="M5" s="5"/>
       <c r="N5" s="5"/>
       <c r="O5" s="5"/>
-      <c r="P5" s="75"/>
+      <c r="P5" s="73"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -2712,7 +2693,7 @@
       <c r="M6" s="5"/>
       <c r="N6" s="5"/>
       <c r="O6" s="5"/>
-      <c r="P6" s="75"/>
+      <c r="P6" s="73"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2730,7 +2711,7 @@
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
       <c r="O7" s="7"/>
-      <c r="P7" s="75"/>
+      <c r="P7" s="73"/>
     </row>
     <row r="8" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2748,7 +2729,7 @@
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>
       <c r="O8" s="7"/>
-      <c r="P8" s="75"/>
+      <c r="P8" s="73"/>
     </row>
     <row r="9" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2783,16 +2764,16 @@
         <v>461</v>
       </c>
       <c r="L9" s="29" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="M9" s="29" t="s">
+        <v>508</v>
+      </c>
+      <c r="N9" s="29" t="s">
         <v>506</v>
       </c>
-      <c r="N9" s="29" t="s">
+      <c r="O9" s="29" t="s">
         <v>507</v>
-      </c>
-      <c r="O9" s="29" t="s">
-        <v>508</v>
       </c>
       <c r="P9" s="56" t="s">
         <v>465</v>
@@ -2832,16 +2813,17 @@
         <v>1</v>
       </c>
       <c r="L10" s="36">
+        <f>K10*10</f>
+        <v>10</v>
+      </c>
+      <c r="M10" s="36">
         <v>12</v>
       </c>
-      <c r="M10" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N10" s="69">
+      <c r="N10" s="67">
         <v>0.21779999999999999</v>
       </c>
-      <c r="O10" s="63">
-        <f>N10*L10</f>
+      <c r="O10" s="62">
+        <f t="shared" ref="O10:O41" si="0">N10*M10</f>
         <v>2.6135999999999999</v>
       </c>
       <c r="P10" s="36"/>
@@ -2849,7 +2831,7 @@
     <row r="11" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="50">
-        <f t="shared" ref="B11:B119" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B119" si="1">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="58" t="s">
@@ -2880,16 +2862,17 @@
         <v>1</v>
       </c>
       <c r="L11" s="38">
+        <f t="shared" ref="L11:L74" si="2">K11*10</f>
+        <v>10</v>
+      </c>
+      <c r="M11" s="38">
         <v>15</v>
       </c>
-      <c r="M11" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N11" s="65">
+      <c r="N11" s="63">
         <v>0.20350000000000001</v>
       </c>
-      <c r="O11" s="65">
-        <f t="shared" ref="O11:O74" si="1">N11*L11</f>
+      <c r="O11" s="63">
+        <f t="shared" si="0"/>
         <v>3.0525000000000002</v>
       </c>
       <c r="P11" s="38"/>
@@ -2928,16 +2911,17 @@
         <v>3</v>
       </c>
       <c r="L12" s="36">
+        <f t="shared" si="2"/>
+        <v>30</v>
+      </c>
+      <c r="M12" s="36">
         <v>100</v>
       </c>
-      <c r="M12" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N12" s="63">
+      <c r="N12" s="62">
         <v>0.10210000000000001</v>
       </c>
-      <c r="O12" s="63">
-        <f t="shared" si="1"/>
+      <c r="O12" s="62">
+        <f t="shared" si="0"/>
         <v>10.210000000000001</v>
       </c>
       <c r="P12" s="36"/>
@@ -2945,7 +2929,7 @@
     <row r="13" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="C13" s="58" t="s">
@@ -2976,16 +2960,17 @@
         <v>5</v>
       </c>
       <c r="L13" s="38">
+        <f t="shared" si="2"/>
+        <v>50</v>
+      </c>
+      <c r="M13" s="38">
         <v>100</v>
       </c>
-      <c r="M13" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N13" s="65">
+      <c r="N13" s="63">
         <v>0.10300000000000001</v>
       </c>
-      <c r="O13" s="65">
-        <f t="shared" si="1"/>
+      <c r="O13" s="63">
+        <f t="shared" si="0"/>
         <v>10.3</v>
       </c>
       <c r="P13" s="38"/>
@@ -3024,16 +3009,17 @@
         <v>7</v>
       </c>
       <c r="L14" s="36">
+        <f t="shared" si="2"/>
+        <v>70</v>
+      </c>
+      <c r="M14" s="36">
         <v>80</v>
       </c>
-      <c r="M14" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N14" s="63">
+      <c r="N14" s="62">
         <v>0.11810000000000001</v>
       </c>
-      <c r="O14" s="63">
-        <f t="shared" si="1"/>
+      <c r="O14" s="62">
+        <f t="shared" si="0"/>
         <v>9.4480000000000004</v>
       </c>
       <c r="P14" s="36"/>
@@ -3041,7 +3027,7 @@
     <row r="15" spans="1:16" ht="180.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="C15" s="58" t="s">
@@ -3072,16 +3058,17 @@
         <v>126</v>
       </c>
       <c r="L15" s="38">
+        <f t="shared" si="2"/>
+        <v>1260</v>
+      </c>
+      <c r="M15" s="38">
         <v>1300</v>
       </c>
-      <c r="M15" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N15" s="65">
+      <c r="N15" s="63">
         <v>0.1009</v>
       </c>
-      <c r="O15" s="65">
-        <f t="shared" si="1"/>
+      <c r="O15" s="63">
+        <f t="shared" si="0"/>
         <v>131.17000000000002</v>
       </c>
       <c r="P15" s="38"/>
@@ -3120,16 +3107,17 @@
         <v>16</v>
       </c>
       <c r="L16" s="36">
+        <f t="shared" si="2"/>
+        <v>160</v>
+      </c>
+      <c r="M16" s="36">
         <v>180</v>
       </c>
-      <c r="M16" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N16" s="63">
+      <c r="N16" s="62">
         <v>0.11420000000000001</v>
       </c>
-      <c r="O16" s="63">
-        <f t="shared" si="1"/>
+      <c r="O16" s="62">
+        <f t="shared" si="0"/>
         <v>20.556000000000001</v>
       </c>
       <c r="P16" s="36"/>
@@ -3137,7 +3125,7 @@
     <row r="17" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="C17" s="58" t="s">
@@ -3168,16 +3156,17 @@
         <v>25</v>
       </c>
       <c r="L17" s="38">
+        <f t="shared" si="2"/>
+        <v>250</v>
+      </c>
+      <c r="M17" s="38">
         <v>280</v>
       </c>
-      <c r="M17" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N17" s="65">
+      <c r="N17" s="63">
         <v>0.11360000000000001</v>
       </c>
-      <c r="O17" s="65">
-        <f t="shared" si="1"/>
+      <c r="O17" s="63">
+        <f t="shared" si="0"/>
         <v>31.808000000000003</v>
       </c>
       <c r="P17" s="38"/>
@@ -3216,16 +3205,17 @@
         <v>27</v>
       </c>
       <c r="L18" s="36">
+        <f t="shared" si="2"/>
+        <v>270</v>
+      </c>
+      <c r="M18" s="36">
         <v>300</v>
       </c>
-      <c r="M18" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N18" s="63">
+      <c r="N18" s="62">
         <v>0.1052</v>
       </c>
-      <c r="O18" s="63">
-        <f t="shared" si="1"/>
+      <c r="O18" s="62">
+        <f t="shared" si="0"/>
         <v>31.560000000000002</v>
       </c>
       <c r="P18" s="36"/>
@@ -3233,7 +3223,7 @@
     <row r="19" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="C19" s="58" t="s">
@@ -3264,16 +3254,17 @@
         <v>9</v>
       </c>
       <c r="L19" s="38">
+        <f t="shared" si="2"/>
+        <v>90</v>
+      </c>
+      <c r="M19" s="38">
         <v>100</v>
       </c>
-      <c r="M19" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N19" s="65">
+      <c r="N19" s="63">
         <v>0.10310000000000001</v>
       </c>
-      <c r="O19" s="65">
-        <f t="shared" si="1"/>
+      <c r="O19" s="63">
+        <f t="shared" si="0"/>
         <v>10.31</v>
       </c>
       <c r="P19" s="38"/>
@@ -3312,16 +3303,17 @@
         <v>4</v>
       </c>
       <c r="L20" s="36">
+        <f t="shared" si="2"/>
+        <v>40</v>
+      </c>
+      <c r="M20" s="36">
         <v>50</v>
       </c>
-      <c r="M20" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N20" s="63">
+      <c r="N20" s="62">
         <v>0.10750000000000001</v>
       </c>
-      <c r="O20" s="63">
-        <f t="shared" si="1"/>
+      <c r="O20" s="62">
+        <f t="shared" si="0"/>
         <v>5.3750000000000009</v>
       </c>
       <c r="P20" s="36"/>
@@ -3329,7 +3321,7 @@
     <row r="21" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="C21" s="58" t="s">
@@ -3360,16 +3352,17 @@
         <v>6</v>
       </c>
       <c r="L21" s="38">
+        <f t="shared" si="2"/>
+        <v>60</v>
+      </c>
+      <c r="M21" s="38">
         <v>100</v>
       </c>
-      <c r="M21" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N21" s="65">
+      <c r="N21" s="63">
         <v>0.10290000000000001</v>
       </c>
-      <c r="O21" s="65">
-        <f t="shared" si="1"/>
+      <c r="O21" s="63">
+        <f t="shared" si="0"/>
         <v>10.290000000000001</v>
       </c>
       <c r="P21" s="38"/>
@@ -3408,16 +3401,17 @@
         <v>1</v>
       </c>
       <c r="L22" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M22" s="36">
         <v>50</v>
       </c>
-      <c r="M22" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N22" s="63">
+      <c r="N22" s="62">
         <v>0.11330000000000001</v>
       </c>
-      <c r="O22" s="63">
-        <f t="shared" si="1"/>
+      <c r="O22" s="62">
+        <f t="shared" si="0"/>
         <v>5.6650000000000009</v>
       </c>
       <c r="P22" s="36"/>
@@ -3425,7 +3419,7 @@
     <row r="23" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>14</v>
       </c>
       <c r="C23" s="58" t="s">
@@ -3456,16 +3450,17 @@
         <v>2</v>
       </c>
       <c r="L23" s="38">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M23" s="38">
         <v>100</v>
       </c>
-      <c r="M23" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N23" s="65">
+      <c r="N23" s="63">
         <v>0.1027</v>
       </c>
-      <c r="O23" s="65">
-        <f t="shared" si="1"/>
+      <c r="O23" s="63">
+        <f t="shared" si="0"/>
         <v>10.27</v>
       </c>
       <c r="P23" s="38"/>
@@ -3504,16 +3499,17 @@
         <v>2</v>
       </c>
       <c r="L24" s="36">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M24" s="36">
         <v>50</v>
       </c>
-      <c r="M24" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N24" s="63">
+      <c r="N24" s="62">
         <v>0.115</v>
       </c>
-      <c r="O24" s="63">
-        <f t="shared" si="1"/>
+      <c r="O24" s="62">
+        <f t="shared" si="0"/>
         <v>5.75</v>
       </c>
       <c r="P24" s="36"/>
@@ -3521,7 +3517,7 @@
     <row r="25" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>16</v>
       </c>
       <c r="C25" s="58" t="s">
@@ -3552,16 +3548,17 @@
         <v>10</v>
       </c>
       <c r="L25" s="38">
+        <f t="shared" si="2"/>
+        <v>100</v>
+      </c>
+      <c r="M25" s="38">
         <v>150</v>
       </c>
-      <c r="M25" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N25" s="65">
+      <c r="N25" s="63">
         <v>0.10700000000000001</v>
       </c>
-      <c r="O25" s="65">
-        <f t="shared" si="1"/>
+      <c r="O25" s="63">
+        <f t="shared" si="0"/>
         <v>16.05</v>
       </c>
       <c r="P25" s="38"/>
@@ -3600,16 +3597,17 @@
         <v>4</v>
       </c>
       <c r="L26" s="36">
+        <f t="shared" si="2"/>
+        <v>40</v>
+      </c>
+      <c r="M26" s="36">
         <v>100</v>
       </c>
-      <c r="M26" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N26" s="63">
+      <c r="N26" s="62">
         <v>0.1028</v>
       </c>
-      <c r="O26" s="63">
-        <f t="shared" si="1"/>
+      <c r="O26" s="62">
+        <f t="shared" si="0"/>
         <v>10.280000000000001</v>
       </c>
       <c r="P26" s="36"/>
@@ -3617,7 +3615,7 @@
     <row r="27" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>18</v>
       </c>
       <c r="C27" s="58" t="s">
@@ -3648,16 +3646,17 @@
         <v>8</v>
       </c>
       <c r="L27" s="38">
+        <f t="shared" si="2"/>
+        <v>80</v>
+      </c>
+      <c r="M27" s="38">
         <v>100</v>
       </c>
-      <c r="M27" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N27" s="65">
+      <c r="N27" s="63">
         <v>0.1202</v>
       </c>
-      <c r="O27" s="65">
-        <f t="shared" si="1"/>
+      <c r="O27" s="63">
+        <f t="shared" si="0"/>
         <v>12.02</v>
       </c>
       <c r="P27" s="38"/>
@@ -3696,16 +3695,17 @@
         <v>6</v>
       </c>
       <c r="L28" s="36">
+        <f t="shared" si="2"/>
+        <v>60</v>
+      </c>
+      <c r="M28" s="36">
         <v>100</v>
       </c>
-      <c r="M28" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N28" s="63">
+      <c r="N28" s="62">
         <v>0.11950000000000001</v>
       </c>
-      <c r="O28" s="63">
-        <f t="shared" si="1"/>
+      <c r="O28" s="62">
+        <f t="shared" si="0"/>
         <v>11.950000000000001</v>
       </c>
       <c r="P28" s="36"/>
@@ -3713,7 +3713,7 @@
     <row r="29" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>20</v>
       </c>
       <c r="C29" s="58" t="s">
@@ -3744,16 +3744,17 @@
         <v>3</v>
       </c>
       <c r="L29" s="38">
+        <f t="shared" si="2"/>
+        <v>30</v>
+      </c>
+      <c r="M29" s="38">
         <v>40</v>
       </c>
-      <c r="M29" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N29" s="65">
+      <c r="N29" s="63">
         <v>0.1477</v>
       </c>
-      <c r="O29" s="65">
-        <f t="shared" si="1"/>
+      <c r="O29" s="63">
+        <f t="shared" si="0"/>
         <v>5.9079999999999995</v>
       </c>
       <c r="P29" s="38"/>
@@ -3792,16 +3793,17 @@
         <v>8</v>
       </c>
       <c r="L30" s="36">
+        <f t="shared" si="2"/>
+        <v>80</v>
+      </c>
+      <c r="M30" s="36">
         <v>100</v>
       </c>
-      <c r="M30" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N30" s="63">
+      <c r="N30" s="62">
         <v>0.12920000000000001</v>
       </c>
-      <c r="O30" s="63">
-        <f t="shared" si="1"/>
+      <c r="O30" s="62">
+        <f t="shared" si="0"/>
         <v>12.920000000000002</v>
       </c>
       <c r="P30" s="36"/>
@@ -3809,7 +3811,7 @@
     <row r="31" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>22</v>
       </c>
       <c r="C31" s="58" t="s">
@@ -3840,16 +3842,17 @@
         <v>5</v>
       </c>
       <c r="L31" s="38">
+        <f t="shared" si="2"/>
+        <v>50</v>
+      </c>
+      <c r="M31" s="38">
         <v>55</v>
       </c>
-      <c r="M31" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N31" s="65">
+      <c r="N31" s="63">
         <v>0.21610000000000001</v>
       </c>
-      <c r="O31" s="65">
-        <f t="shared" si="1"/>
+      <c r="O31" s="63">
+        <f t="shared" si="0"/>
         <v>11.8855</v>
       </c>
       <c r="P31" s="38"/>
@@ -3888,16 +3891,17 @@
         <v>3</v>
       </c>
       <c r="L32" s="36">
+        <f t="shared" si="2"/>
+        <v>30</v>
+      </c>
+      <c r="M32" s="36">
         <v>35</v>
       </c>
-      <c r="M32" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N32" s="63">
+      <c r="N32" s="62">
         <v>0.18359999999999999</v>
       </c>
-      <c r="O32" s="63">
-        <f t="shared" si="1"/>
+      <c r="O32" s="62">
+        <f t="shared" si="0"/>
         <v>6.4259999999999993</v>
       </c>
       <c r="P32" s="36"/>
@@ -3905,7 +3909,7 @@
     <row r="33" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>24</v>
       </c>
       <c r="C33" s="58" t="s">
@@ -3936,16 +3940,17 @@
         <v>1</v>
       </c>
       <c r="L33" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M33" s="38">
         <v>12</v>
       </c>
-      <c r="M33" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N33" s="65">
+      <c r="N33" s="63">
         <v>0.41849999999999998</v>
       </c>
-      <c r="O33" s="65">
-        <f t="shared" si="1"/>
+      <c r="O33" s="63">
+        <f t="shared" si="0"/>
         <v>5.0220000000000002</v>
       </c>
       <c r="P33" s="38"/>
@@ -3984,16 +3989,17 @@
         <v>1</v>
       </c>
       <c r="L34" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M34" s="36">
         <v>20</v>
       </c>
-      <c r="M34" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N34" s="63">
+      <c r="N34" s="62">
         <v>0.13620000000000002</v>
       </c>
-      <c r="O34" s="63">
-        <f t="shared" si="1"/>
+      <c r="O34" s="62">
+        <f t="shared" si="0"/>
         <v>2.7240000000000002</v>
       </c>
       <c r="P34" s="36"/>
@@ -4001,7 +4007,7 @@
     <row r="35" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>26</v>
       </c>
       <c r="C35" s="58" t="s">
@@ -4032,16 +4038,17 @@
         <v>1</v>
       </c>
       <c r="L35" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M35" s="38">
         <v>20</v>
       </c>
-      <c r="M35" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N35" s="65">
+      <c r="N35" s="63">
         <v>0.14900000000000002</v>
       </c>
-      <c r="O35" s="65">
-        <f t="shared" si="1"/>
+      <c r="O35" s="63">
+        <f t="shared" si="0"/>
         <v>2.9800000000000004</v>
       </c>
       <c r="P35" s="38"/>
@@ -4080,16 +4087,17 @@
         <v>1</v>
       </c>
       <c r="L36" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M36" s="36">
         <v>20</v>
       </c>
-      <c r="M36" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N36" s="63">
+      <c r="N36" s="62">
         <v>0.12820000000000001</v>
       </c>
-      <c r="O36" s="63">
-        <f t="shared" si="1"/>
+      <c r="O36" s="62">
+        <f t="shared" si="0"/>
         <v>2.5640000000000001</v>
       </c>
       <c r="P36" s="36"/>
@@ -4097,7 +4105,7 @@
     <row r="37" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="C37" s="58" t="s">
@@ -4128,16 +4136,17 @@
         <v>1</v>
       </c>
       <c r="L37" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M37" s="38">
         <v>12</v>
       </c>
-      <c r="M37" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N37" s="65">
+      <c r="N37" s="63">
         <v>0.67669999999999997</v>
       </c>
-      <c r="O37" s="65">
-        <f t="shared" si="1"/>
+      <c r="O37" s="63">
+        <f t="shared" si="0"/>
         <v>8.1204000000000001</v>
       </c>
       <c r="P37" s="38"/>
@@ -4176,16 +4185,17 @@
         <v>1</v>
       </c>
       <c r="L38" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M38" s="36">
         <v>11</v>
       </c>
-      <c r="M38" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N38" s="63">
+      <c r="N38" s="62">
         <v>0.23469999999999999</v>
       </c>
-      <c r="O38" s="63">
-        <f t="shared" si="1"/>
+      <c r="O38" s="62">
+        <f t="shared" si="0"/>
         <v>2.5817000000000001</v>
       </c>
       <c r="P38" s="36"/>
@@ -4193,7 +4203,7 @@
     <row r="39" spans="1:16" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>30</v>
       </c>
       <c r="C39" s="58" t="s">
@@ -4224,16 +4234,17 @@
         <v>1</v>
       </c>
       <c r="L39" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M39" s="38">
         <v>12</v>
       </c>
-      <c r="M39" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N39" s="65">
+      <c r="N39" s="63">
         <v>0.23569999999999999</v>
       </c>
-      <c r="O39" s="65">
-        <f t="shared" si="1"/>
+      <c r="O39" s="63">
+        <f t="shared" si="0"/>
         <v>2.8283999999999998</v>
       </c>
       <c r="P39" s="38"/>
@@ -4272,16 +4283,17 @@
         <v>1</v>
       </c>
       <c r="L40" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M40" s="36">
         <v>11</v>
       </c>
-      <c r="M40" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N40" s="63">
+      <c r="N40" s="62">
         <v>1.8351000000000002</v>
       </c>
-      <c r="O40" s="63">
-        <f t="shared" si="1"/>
+      <c r="O40" s="62">
+        <f t="shared" si="0"/>
         <v>20.186100000000003</v>
       </c>
       <c r="P40" s="36"/>
@@ -4289,7 +4301,7 @@
     <row r="41" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
       <c r="B41" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>32</v>
       </c>
       <c r="C41" s="58" t="s">
@@ -4320,16 +4332,17 @@
         <v>1</v>
       </c>
       <c r="L41" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M41" s="38">
         <v>12</v>
       </c>
-      <c r="M41" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N41" s="65">
+      <c r="N41" s="63">
         <v>0.52870000000000006</v>
       </c>
-      <c r="O41" s="65">
-        <f t="shared" si="1"/>
+      <c r="O41" s="63">
+        <f t="shared" si="0"/>
         <v>6.3444000000000003</v>
       </c>
       <c r="P41" s="38"/>
@@ -4368,16 +4381,17 @@
         <v>2</v>
       </c>
       <c r="L42" s="36">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M42" s="36">
         <v>25</v>
       </c>
-      <c r="M42" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N42" s="63">
+      <c r="N42" s="62">
         <v>0.1875</v>
       </c>
-      <c r="O42" s="63">
-        <f t="shared" si="1"/>
+      <c r="O42" s="62">
+        <f t="shared" ref="O42:O73" si="3">N42*M42</f>
         <v>4.6875</v>
       </c>
       <c r="P42" s="36"/>
@@ -4385,7 +4399,7 @@
     <row r="43" spans="1:16" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>34</v>
       </c>
       <c r="C43" s="58" t="s">
@@ -4416,16 +4430,17 @@
         <v>1</v>
       </c>
       <c r="L43" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M43" s="38">
         <v>20</v>
       </c>
-      <c r="M43" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N43" s="65">
+      <c r="N43" s="63">
         <v>0.1447</v>
       </c>
-      <c r="O43" s="65">
-        <f t="shared" si="1"/>
+      <c r="O43" s="63">
+        <f t="shared" si="3"/>
         <v>2.8940000000000001</v>
       </c>
       <c r="P43" s="38"/>
@@ -4464,16 +4479,17 @@
         <v>1</v>
       </c>
       <c r="L44" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M44" s="36">
         <v>12</v>
       </c>
-      <c r="M44" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N44" s="63">
+      <c r="N44" s="62">
         <v>0.40129999999999999</v>
       </c>
-      <c r="O44" s="63">
-        <f t="shared" si="1"/>
+      <c r="O44" s="62">
+        <f t="shared" si="3"/>
         <v>4.8155999999999999</v>
       </c>
       <c r="P44" s="36"/>
@@ -4481,7 +4497,7 @@
     <row r="45" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
       <c r="B45" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>36</v>
       </c>
       <c r="C45" s="58" t="s">
@@ -4512,16 +4528,17 @@
         <v>1</v>
       </c>
       <c r="L45" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M45" s="38">
         <v>12</v>
       </c>
-      <c r="M45" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N45" s="65">
+      <c r="N45" s="63">
         <v>0.76449999999999996</v>
       </c>
-      <c r="O45" s="65">
-        <f t="shared" si="1"/>
+      <c r="O45" s="63">
+        <f t="shared" si="3"/>
         <v>9.1739999999999995</v>
       </c>
       <c r="P45" s="38"/>
@@ -4560,16 +4577,17 @@
         <v>1</v>
       </c>
       <c r="L46" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M46" s="36">
         <v>12</v>
       </c>
-      <c r="M46" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N46" s="63">
+      <c r="N46" s="62">
         <v>0.27039999999999997</v>
       </c>
-      <c r="O46" s="63">
-        <f t="shared" si="1"/>
+      <c r="O46" s="62">
+        <f t="shared" si="3"/>
         <v>3.2447999999999997</v>
       </c>
       <c r="P46" s="36"/>
@@ -4577,7 +4595,7 @@
     <row r="47" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
       <c r="B47" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>38</v>
       </c>
       <c r="C47" s="58" t="s">
@@ -4608,16 +4626,17 @@
         <v>1</v>
       </c>
       <c r="L47" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M47" s="38">
         <v>20</v>
       </c>
-      <c r="M47" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N47" s="65">
+      <c r="N47" s="63">
         <v>0.1515</v>
       </c>
-      <c r="O47" s="65">
-        <f t="shared" si="1"/>
+      <c r="O47" s="63">
+        <f t="shared" si="3"/>
         <v>3.03</v>
       </c>
       <c r="P47" s="38"/>
@@ -4656,16 +4675,17 @@
         <v>2</v>
       </c>
       <c r="L48" s="36">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M48" s="36">
         <v>30</v>
       </c>
-      <c r="M48" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N48" s="63">
+      <c r="N48" s="62">
         <v>0.16090000000000002</v>
       </c>
-      <c r="O48" s="63">
-        <f t="shared" si="1"/>
+      <c r="O48" s="62">
+        <f t="shared" si="3"/>
         <v>4.8270000000000008</v>
       </c>
       <c r="P48" s="36"/>
@@ -4673,7 +4693,7 @@
     <row r="49" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
       <c r="B49" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>40</v>
       </c>
       <c r="C49" s="58" t="s">
@@ -4704,16 +4724,17 @@
         <v>1</v>
       </c>
       <c r="L49" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M49" s="38">
         <v>12</v>
       </c>
-      <c r="M49" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N49" s="65">
+      <c r="N49" s="63">
         <v>0.24030000000000001</v>
       </c>
-      <c r="O49" s="65">
-        <f t="shared" si="1"/>
+      <c r="O49" s="63">
+        <f t="shared" si="3"/>
         <v>2.8836000000000004</v>
       </c>
       <c r="P49" s="38"/>
@@ -4752,16 +4773,17 @@
         <v>2</v>
       </c>
       <c r="L50" s="36">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M50" s="36">
         <v>30</v>
       </c>
-      <c r="M50" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N50" s="63">
+      <c r="N50" s="62">
         <v>0.14380000000000001</v>
       </c>
-      <c r="O50" s="63">
-        <f t="shared" si="1"/>
+      <c r="O50" s="62">
+        <f t="shared" si="3"/>
         <v>4.3140000000000001</v>
       </c>
       <c r="P50" s="36"/>
@@ -4769,7 +4791,7 @@
     <row r="51" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1"/>
       <c r="B51" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>42</v>
       </c>
       <c r="C51" s="58" t="s">
@@ -4800,16 +4822,17 @@
         <v>2</v>
       </c>
       <c r="L51" s="38">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M51" s="38">
         <v>22</v>
       </c>
-      <c r="M51" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N51" s="65">
+      <c r="N51" s="63">
         <v>0.23650000000000002</v>
       </c>
-      <c r="O51" s="65">
-        <f t="shared" si="1"/>
+      <c r="O51" s="63">
+        <f t="shared" si="3"/>
         <v>5.2030000000000003</v>
       </c>
       <c r="P51" s="38"/>
@@ -4848,16 +4871,17 @@
         <v>2</v>
       </c>
       <c r="L52" s="36">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M52" s="36">
         <v>22</v>
       </c>
-      <c r="M52" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N52" s="63">
+      <c r="N52" s="62">
         <v>0.248</v>
       </c>
-      <c r="O52" s="63">
-        <f t="shared" si="1"/>
+      <c r="O52" s="62">
+        <f t="shared" si="3"/>
         <v>5.4559999999999995</v>
       </c>
       <c r="P52" s="36"/>
@@ -4865,7 +4889,7 @@
     <row r="53" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1"/>
       <c r="B53" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>44</v>
       </c>
       <c r="C53" s="58" t="s">
@@ -4896,16 +4920,17 @@
         <v>1</v>
       </c>
       <c r="L53" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M53" s="38">
         <v>20</v>
       </c>
-      <c r="M53" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N53" s="65">
+      <c r="N53" s="63">
         <v>0.1706</v>
       </c>
-      <c r="O53" s="65">
-        <f t="shared" si="1"/>
+      <c r="O53" s="63">
+        <f t="shared" si="3"/>
         <v>3.4119999999999999</v>
       </c>
       <c r="P53" s="38"/>
@@ -4944,16 +4969,17 @@
         <v>1</v>
       </c>
       <c r="L54" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M54" s="36">
         <v>100</v>
       </c>
-      <c r="M54" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N54" s="63">
+      <c r="N54" s="62">
         <v>0.10310000000000001</v>
       </c>
-      <c r="O54" s="63">
-        <f t="shared" si="1"/>
+      <c r="O54" s="62">
+        <f t="shared" si="3"/>
         <v>10.31</v>
       </c>
       <c r="P54" s="36"/>
@@ -4961,7 +4987,7 @@
     <row r="55" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
       <c r="B55" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>46</v>
       </c>
       <c r="C55" s="58" t="s">
@@ -4992,16 +5018,17 @@
         <v>1</v>
       </c>
       <c r="L55" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M55" s="38">
         <v>20</v>
       </c>
-      <c r="M55" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N55" s="65">
+      <c r="N55" s="63">
         <v>0.15620000000000001</v>
       </c>
-      <c r="O55" s="65">
-        <f t="shared" si="1"/>
+      <c r="O55" s="63">
+        <f t="shared" si="3"/>
         <v>3.1240000000000001</v>
       </c>
       <c r="P55" s="38"/>
@@ -5040,16 +5067,17 @@
         <v>1</v>
       </c>
       <c r="L56" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M56" s="36">
         <v>50</v>
       </c>
-      <c r="M56" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N56" s="63">
+      <c r="N56" s="62">
         <v>0.1163</v>
       </c>
-      <c r="O56" s="63">
-        <f t="shared" si="1"/>
+      <c r="O56" s="62">
+        <f t="shared" si="3"/>
         <v>5.8150000000000004</v>
       </c>
       <c r="P56" s="36"/>
@@ -5057,7 +5085,7 @@
     <row r="57" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
       <c r="B57" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>48</v>
       </c>
       <c r="C57" s="58" t="s">
@@ -5088,16 +5116,17 @@
         <v>1</v>
       </c>
       <c r="L57" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M57" s="38">
         <v>20</v>
       </c>
-      <c r="M57" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N57" s="65">
+      <c r="N57" s="63">
         <v>0.13540000000000002</v>
       </c>
-      <c r="O57" s="65">
-        <f t="shared" si="1"/>
+      <c r="O57" s="63">
+        <f t="shared" si="3"/>
         <v>2.7080000000000002</v>
       </c>
       <c r="P57" s="38"/>
@@ -5136,16 +5165,17 @@
         <v>1</v>
       </c>
       <c r="L58" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M58" s="36">
         <v>20</v>
       </c>
-      <c r="M58" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N58" s="63">
+      <c r="N58" s="62">
         <v>0.13520000000000001</v>
       </c>
-      <c r="O58" s="63">
-        <f t="shared" si="1"/>
+      <c r="O58" s="62">
+        <f t="shared" si="3"/>
         <v>2.7040000000000002</v>
       </c>
       <c r="P58" s="36"/>
@@ -5153,7 +5183,7 @@
     <row r="59" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1"/>
       <c r="B59" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>50</v>
       </c>
       <c r="C59" s="58" t="s">
@@ -5184,14 +5214,17 @@
         <v>1</v>
       </c>
       <c r="L59" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M59" s="38">
         <v>50</v>
       </c>
-      <c r="M59" s="64"/>
-      <c r="N59" s="65">
+      <c r="N59" s="63">
         <v>0.1159</v>
       </c>
-      <c r="O59" s="65">
-        <f t="shared" si="1"/>
+      <c r="O59" s="63">
+        <f t="shared" si="3"/>
         <v>5.7949999999999999</v>
       </c>
       <c r="P59" s="38"/>
@@ -5229,16 +5262,17 @@
       <c r="K60" s="37">
         <v>28</v>
       </c>
-      <c r="L60" s="36" t="s">
-        <v>480</v>
-      </c>
-      <c r="M60" s="62" t="s">
-        <v>480</v>
-      </c>
-      <c r="N60" s="63">
+      <c r="L60" s="36">
+        <f t="shared" si="2"/>
+        <v>280</v>
+      </c>
+      <c r="M60" s="36" t="s">
+        <v>480</v>
+      </c>
+      <c r="N60" s="62">
         <v>0</v>
       </c>
-      <c r="O60" s="63" t="s">
+      <c r="O60" s="62" t="s">
         <v>480</v>
       </c>
       <c r="P60" s="36"/>
@@ -5246,7 +5280,7 @@
     <row r="61" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="1"/>
       <c r="B61" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>52</v>
       </c>
       <c r="C61" s="58" t="s">
@@ -5277,16 +5311,17 @@
         <v>10</v>
       </c>
       <c r="L61" s="38">
+        <f t="shared" si="2"/>
+        <v>100</v>
+      </c>
+      <c r="M61" s="38">
         <v>150</v>
       </c>
-      <c r="M61" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N61" s="65">
+      <c r="N61" s="63">
         <v>0.11360000000000001</v>
       </c>
-      <c r="O61" s="65">
-        <f t="shared" si="1"/>
+      <c r="O61" s="63">
+        <f t="shared" ref="O61:O98" si="4">N61*M61</f>
         <v>17.040000000000003</v>
       </c>
       <c r="P61" s="38"/>
@@ -5325,16 +5360,17 @@
         <v>1</v>
       </c>
       <c r="L62" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M62" s="36">
         <v>20</v>
       </c>
-      <c r="M62" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N62" s="63">
+      <c r="N62" s="62">
         <v>0.13150000000000001</v>
       </c>
-      <c r="O62" s="63">
-        <f t="shared" si="1"/>
+      <c r="O62" s="62">
+        <f t="shared" si="4"/>
         <v>2.63</v>
       </c>
       <c r="P62" s="36"/>
@@ -5342,7 +5378,7 @@
     <row r="63" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1"/>
       <c r="B63" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>54</v>
       </c>
       <c r="C63" s="58" t="s">
@@ -5373,16 +5409,17 @@
         <v>1</v>
       </c>
       <c r="L63" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M63" s="38">
         <v>50</v>
       </c>
-      <c r="M63" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N63" s="65">
+      <c r="N63" s="63">
         <v>0.11650000000000001</v>
       </c>
-      <c r="O63" s="65">
-        <f t="shared" si="1"/>
+      <c r="O63" s="63">
+        <f t="shared" si="4"/>
         <v>5.8250000000000002</v>
       </c>
       <c r="P63" s="38"/>
@@ -5421,16 +5458,17 @@
         <v>1</v>
       </c>
       <c r="L64" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M64" s="36">
         <v>20</v>
       </c>
-      <c r="M64" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N64" s="63">
+      <c r="N64" s="62">
         <v>0.13670000000000002</v>
       </c>
-      <c r="O64" s="63">
-        <f t="shared" si="1"/>
+      <c r="O64" s="62">
+        <f t="shared" si="4"/>
         <v>2.7340000000000004</v>
       </c>
       <c r="P64" s="36"/>
@@ -5438,7 +5476,7 @@
     <row r="65" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="1"/>
       <c r="B65" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>56</v>
       </c>
       <c r="C65" s="58" t="s">
@@ -5469,16 +5507,17 @@
         <v>5</v>
       </c>
       <c r="L65" s="38">
+        <f t="shared" si="2"/>
+        <v>50</v>
+      </c>
+      <c r="M65" s="38">
         <v>60</v>
       </c>
-      <c r="M65" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N65" s="65">
+      <c r="N65" s="63">
         <v>0.12050000000000001</v>
       </c>
-      <c r="O65" s="65">
-        <f t="shared" si="1"/>
+      <c r="O65" s="63">
+        <f t="shared" si="4"/>
         <v>7.23</v>
       </c>
       <c r="P65" s="38"/>
@@ -5517,16 +5556,17 @@
         <v>3</v>
       </c>
       <c r="L66" s="36">
+        <f t="shared" si="2"/>
+        <v>30</v>
+      </c>
+      <c r="M66" s="36">
         <v>40</v>
       </c>
-      <c r="M66" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N66" s="63">
+      <c r="N66" s="62">
         <v>0.13140000000000002</v>
       </c>
-      <c r="O66" s="63">
-        <f t="shared" si="1"/>
+      <c r="O66" s="62">
+        <f t="shared" si="4"/>
         <v>5.2560000000000002</v>
       </c>
       <c r="P66" s="36"/>
@@ -5534,7 +5574,7 @@
     <row r="67" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="1"/>
       <c r="B67" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>58</v>
       </c>
       <c r="C67" s="58" t="s">
@@ -5565,16 +5605,17 @@
         <v>1</v>
       </c>
       <c r="L67" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M67" s="38">
         <v>20</v>
       </c>
-      <c r="M67" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N67" s="65">
+      <c r="N67" s="63">
         <v>0.14960000000000001</v>
       </c>
-      <c r="O67" s="65">
-        <f t="shared" si="1"/>
+      <c r="O67" s="63">
+        <f t="shared" si="4"/>
         <v>2.992</v>
       </c>
       <c r="P67" s="38"/>
@@ -5613,16 +5654,17 @@
         <v>37</v>
       </c>
       <c r="L68" s="36">
+        <f t="shared" si="2"/>
+        <v>370</v>
+      </c>
+      <c r="M68" s="36">
         <v>400</v>
       </c>
-      <c r="M68" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N68" s="63">
+      <c r="N68" s="62">
         <v>0.1017</v>
       </c>
-      <c r="O68" s="63">
-        <f t="shared" si="1"/>
+      <c r="O68" s="62">
+        <f t="shared" si="4"/>
         <v>40.68</v>
       </c>
       <c r="P68" s="36"/>
@@ -5630,7 +5672,7 @@
     <row r="69" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="1"/>
       <c r="B69" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>60</v>
       </c>
       <c r="C69" s="58" t="s">
@@ -5661,16 +5703,17 @@
         <v>6</v>
       </c>
       <c r="L69" s="38">
+        <f t="shared" si="2"/>
+        <v>60</v>
+      </c>
+      <c r="M69" s="38">
         <v>80</v>
       </c>
-      <c r="M69" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N69" s="65">
+      <c r="N69" s="63">
         <v>0.13270000000000001</v>
       </c>
-      <c r="O69" s="65">
-        <f t="shared" si="1"/>
+      <c r="O69" s="63">
+        <f t="shared" si="4"/>
         <v>10.616000000000001</v>
       </c>
       <c r="P69" s="38"/>
@@ -5709,16 +5752,17 @@
         <v>3</v>
       </c>
       <c r="L70" s="36">
+        <f t="shared" si="2"/>
+        <v>30</v>
+      </c>
+      <c r="M70" s="36">
         <v>50</v>
       </c>
-      <c r="M70" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N70" s="63">
+      <c r="N70" s="62">
         <v>0.11330000000000001</v>
       </c>
-      <c r="O70" s="63">
-        <f t="shared" si="1"/>
+      <c r="O70" s="62">
+        <f t="shared" si="4"/>
         <v>5.6650000000000009</v>
       </c>
       <c r="P70" s="36"/>
@@ -5726,7 +5770,7 @@
     <row r="71" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="1"/>
       <c r="B71" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>62</v>
       </c>
       <c r="C71" s="58" t="s">
@@ -5757,16 +5801,17 @@
         <v>1</v>
       </c>
       <c r="L71" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M71" s="38">
         <v>20</v>
       </c>
-      <c r="M71" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N71" s="65">
+      <c r="N71" s="63">
         <v>0.12590000000000001</v>
       </c>
-      <c r="O71" s="65">
-        <f t="shared" si="1"/>
+      <c r="O71" s="63">
+        <f t="shared" si="4"/>
         <v>2.5180000000000002</v>
       </c>
       <c r="P71" s="38"/>
@@ -5805,16 +5850,17 @@
         <v>1</v>
       </c>
       <c r="L72" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M72" s="36">
         <v>20</v>
       </c>
-      <c r="M72" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N72" s="63">
+      <c r="N72" s="62">
         <v>0.12859999999999999</v>
       </c>
-      <c r="O72" s="63">
-        <f t="shared" si="1"/>
+      <c r="O72" s="62">
+        <f t="shared" si="4"/>
         <v>2.5720000000000001</v>
       </c>
       <c r="P72" s="36"/>
@@ -5822,7 +5868,7 @@
     <row r="73" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="1"/>
       <c r="B73" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>64</v>
       </c>
       <c r="C73" s="58" t="s">
@@ -5853,16 +5899,17 @@
         <v>1</v>
       </c>
       <c r="L73" s="38">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M73" s="38">
         <v>100</v>
       </c>
-      <c r="M73" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N73" s="65">
+      <c r="N73" s="63">
         <v>0.1014</v>
       </c>
-      <c r="O73" s="65">
-        <f t="shared" si="1"/>
+      <c r="O73" s="63">
+        <f t="shared" si="4"/>
         <v>10.14</v>
       </c>
       <c r="P73" s="38"/>
@@ -5901,16 +5948,17 @@
         <v>1</v>
       </c>
       <c r="L74" s="36">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M74" s="36">
         <v>100</v>
       </c>
-      <c r="M74" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N74" s="63">
+      <c r="N74" s="62">
         <v>0.10120000000000001</v>
       </c>
-      <c r="O74" s="63">
-        <f t="shared" si="1"/>
+      <c r="O74" s="62">
+        <f t="shared" si="4"/>
         <v>10.120000000000001</v>
       </c>
       <c r="P74" s="36"/>
@@ -5918,7 +5966,7 @@
     <row r="75" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="1"/>
       <c r="B75" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>66</v>
       </c>
       <c r="C75" s="58" t="s">
@@ -5949,16 +5997,17 @@
         <v>1</v>
       </c>
       <c r="L75" s="38">
+        <f t="shared" ref="L75:L119" si="5">K75*10</f>
+        <v>10</v>
+      </c>
+      <c r="M75" s="38">
         <v>100</v>
       </c>
-      <c r="M75" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N75" s="65">
+      <c r="N75" s="63">
         <v>0.10110000000000001</v>
       </c>
-      <c r="O75" s="65">
-        <f t="shared" ref="O75:O119" si="2">N75*L75</f>
+      <c r="O75" s="63">
+        <f t="shared" si="4"/>
         <v>10.110000000000001</v>
       </c>
       <c r="P75" s="38"/>
@@ -5997,16 +6046,17 @@
         <v>1</v>
       </c>
       <c r="L76" s="36">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M76" s="36">
         <v>20</v>
       </c>
-      <c r="M76" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N76" s="63">
+      <c r="N76" s="62">
         <v>0.12590000000000001</v>
       </c>
-      <c r="O76" s="63">
-        <f t="shared" si="2"/>
+      <c r="O76" s="62">
+        <f t="shared" si="4"/>
         <v>2.5180000000000002</v>
       </c>
       <c r="P76" s="36"/>
@@ -6014,7 +6064,7 @@
     <row r="77" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="1"/>
       <c r="B77" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>68</v>
       </c>
       <c r="C77" s="58" t="s">
@@ -6045,16 +6095,17 @@
         <v>6</v>
       </c>
       <c r="L77" s="38">
+        <f t="shared" si="5"/>
+        <v>60</v>
+      </c>
+      <c r="M77" s="38">
         <v>100</v>
       </c>
-      <c r="M77" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N77" s="65">
+      <c r="N77" s="63">
         <v>0.1013</v>
       </c>
-      <c r="O77" s="65">
-        <f t="shared" si="2"/>
+      <c r="O77" s="63">
+        <f t="shared" si="4"/>
         <v>10.130000000000001</v>
       </c>
       <c r="P77" s="38"/>
@@ -6093,16 +6144,17 @@
         <v>10</v>
       </c>
       <c r="L78" s="36">
+        <f t="shared" si="5"/>
+        <v>100</v>
+      </c>
+      <c r="M78" s="36">
         <v>200</v>
       </c>
-      <c r="M78" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N78" s="63">
+      <c r="N78" s="62">
         <v>0.10100000000000001</v>
       </c>
-      <c r="O78" s="63">
-        <f t="shared" si="2"/>
+      <c r="O78" s="62">
+        <f t="shared" si="4"/>
         <v>20.200000000000003</v>
       </c>
       <c r="P78" s="36"/>
@@ -6110,7 +6162,7 @@
     <row r="79" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="1"/>
       <c r="B79" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>70</v>
       </c>
       <c r="C79" s="58" t="s">
@@ -6141,16 +6193,17 @@
         <v>1</v>
       </c>
       <c r="L79" s="38">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M79" s="38">
         <v>100</v>
       </c>
-      <c r="M79" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N79" s="65">
+      <c r="N79" s="63">
         <v>0.10310000000000001</v>
       </c>
-      <c r="O79" s="65">
-        <f t="shared" si="2"/>
+      <c r="O79" s="63">
+        <f t="shared" si="4"/>
         <v>10.31</v>
       </c>
       <c r="P79" s="38"/>
@@ -6189,16 +6242,17 @@
         <v>3</v>
       </c>
       <c r="L80" s="36">
+        <f t="shared" si="5"/>
+        <v>30</v>
+      </c>
+      <c r="M80" s="36">
         <v>100</v>
       </c>
-      <c r="M80" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N80" s="63">
+      <c r="N80" s="62">
         <v>0.1009</v>
       </c>
-      <c r="O80" s="63">
-        <f t="shared" si="2"/>
+      <c r="O80" s="62">
+        <f t="shared" si="4"/>
         <v>10.09</v>
       </c>
       <c r="P80" s="36"/>
@@ -6206,7 +6260,7 @@
     <row r="81" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="1"/>
       <c r="B81" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>72</v>
       </c>
       <c r="C81" s="58" t="s">
@@ -6237,16 +6291,17 @@
         <v>1</v>
       </c>
       <c r="L81" s="38">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M81" s="38">
         <v>20</v>
       </c>
-      <c r="M81" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N81" s="65">
+      <c r="N81" s="63">
         <v>0.11940000000000001</v>
       </c>
-      <c r="O81" s="65">
-        <f t="shared" si="2"/>
+      <c r="O81" s="63">
+        <f t="shared" si="4"/>
         <v>2.3879999999999999</v>
       </c>
       <c r="P81" s="38"/>
@@ -6285,16 +6340,17 @@
         <v>1</v>
       </c>
       <c r="L82" s="36">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M82" s="36">
         <v>100</v>
       </c>
-      <c r="M82" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N82" s="63">
+      <c r="N82" s="62">
         <v>0.10200000000000001</v>
       </c>
-      <c r="O82" s="63">
-        <f t="shared" si="2"/>
+      <c r="O82" s="62">
+        <f t="shared" si="4"/>
         <v>10.200000000000001</v>
       </c>
       <c r="P82" s="36"/>
@@ -6302,7 +6358,7 @@
     <row r="83" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A83" s="1"/>
       <c r="B83" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>74</v>
       </c>
       <c r="C83" s="58" t="s">
@@ -6333,16 +6389,17 @@
         <v>10</v>
       </c>
       <c r="L83" s="38">
+        <f t="shared" si="5"/>
+        <v>100</v>
+      </c>
+      <c r="M83" s="38">
         <v>200</v>
       </c>
-      <c r="M83" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N83" s="65">
+      <c r="N83" s="63">
         <v>0.1008</v>
       </c>
-      <c r="O83" s="65">
-        <f t="shared" si="2"/>
+      <c r="O83" s="63">
+        <f t="shared" si="4"/>
         <v>20.16</v>
       </c>
       <c r="P83" s="38"/>
@@ -6381,16 +6438,17 @@
         <v>1</v>
       </c>
       <c r="L84" s="36">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M84" s="36">
         <v>50</v>
       </c>
-      <c r="M84" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N84" s="63">
+      <c r="N84" s="62">
         <v>0.10680000000000001</v>
       </c>
-      <c r="O84" s="63">
-        <f t="shared" si="2"/>
+      <c r="O84" s="62">
+        <f t="shared" si="4"/>
         <v>5.34</v>
       </c>
       <c r="P84" s="36"/>
@@ -6398,7 +6456,7 @@
     <row r="85" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A85" s="1"/>
       <c r="B85" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>76</v>
       </c>
       <c r="C85" s="58" t="s">
@@ -6429,16 +6487,17 @@
         <v>8</v>
       </c>
       <c r="L85" s="38">
+        <f t="shared" si="5"/>
+        <v>80</v>
+      </c>
+      <c r="M85" s="38">
         <v>100</v>
       </c>
-      <c r="M85" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N85" s="65">
+      <c r="N85" s="63">
         <v>0.11430000000000001</v>
       </c>
-      <c r="O85" s="65">
-        <f t="shared" si="2"/>
+      <c r="O85" s="63">
+        <f t="shared" si="4"/>
         <v>11.430000000000001</v>
       </c>
       <c r="P85" s="38"/>
@@ -6477,16 +6536,17 @@
         <v>3</v>
       </c>
       <c r="L86" s="36">
+        <f t="shared" si="5"/>
+        <v>30</v>
+      </c>
+      <c r="M86" s="36">
         <v>100</v>
       </c>
-      <c r="M86" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N86" s="63">
+      <c r="N86" s="62">
         <v>0.10300000000000001</v>
       </c>
-      <c r="O86" s="63">
-        <f t="shared" si="2"/>
+      <c r="O86" s="62">
+        <f t="shared" si="4"/>
         <v>10.3</v>
       </c>
       <c r="P86" s="36"/>
@@ -6494,7 +6554,7 @@
     <row r="87" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="1"/>
       <c r="B87" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>78</v>
       </c>
       <c r="C87" s="58" t="s">
@@ -6525,16 +6585,17 @@
         <v>2</v>
       </c>
       <c r="L87" s="38">
+        <f t="shared" si="5"/>
+        <v>20</v>
+      </c>
+      <c r="M87" s="38">
         <v>40</v>
       </c>
-      <c r="M87" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N87" s="65">
+      <c r="N87" s="63">
         <v>0.12570000000000001</v>
       </c>
-      <c r="O87" s="65">
-        <f t="shared" si="2"/>
+      <c r="O87" s="63">
+        <f t="shared" si="4"/>
         <v>5.0280000000000005</v>
       </c>
       <c r="P87" s="38"/>
@@ -6573,16 +6634,17 @@
         <v>1</v>
       </c>
       <c r="L88" s="36">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M88" s="36">
         <v>100</v>
       </c>
-      <c r="M88" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N88" s="63">
+      <c r="N88" s="62">
         <v>0.10400000000000001</v>
       </c>
-      <c r="O88" s="63">
-        <f t="shared" si="2"/>
+      <c r="O88" s="62">
+        <f t="shared" si="4"/>
         <v>10.4</v>
       </c>
       <c r="P88" s="36"/>
@@ -6590,7 +6652,7 @@
     <row r="89" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A89" s="1"/>
       <c r="B89" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>80</v>
       </c>
       <c r="C89" s="58" t="s">
@@ -6621,16 +6683,17 @@
         <v>3</v>
       </c>
       <c r="L89" s="38">
+        <f t="shared" si="5"/>
+        <v>30</v>
+      </c>
+      <c r="M89" s="38">
         <v>100</v>
       </c>
-      <c r="M89" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N89" s="65">
+      <c r="N89" s="63">
         <v>0.10110000000000001</v>
       </c>
-      <c r="O89" s="65">
-        <f t="shared" si="2"/>
+      <c r="O89" s="63">
+        <f t="shared" si="4"/>
         <v>10.110000000000001</v>
       </c>
       <c r="P89" s="38"/>
@@ -6669,16 +6732,17 @@
         <v>2</v>
       </c>
       <c r="L90" s="36">
+        <f t="shared" si="5"/>
+        <v>20</v>
+      </c>
+      <c r="M90" s="36">
         <v>100</v>
       </c>
-      <c r="M90" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N90" s="63">
+      <c r="N90" s="62">
         <v>0.10110000000000001</v>
       </c>
-      <c r="O90" s="63">
-        <f t="shared" si="2"/>
+      <c r="O90" s="62">
+        <f t="shared" si="4"/>
         <v>10.110000000000001</v>
       </c>
       <c r="P90" s="36"/>
@@ -6686,7 +6750,7 @@
     <row r="91" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A91" s="1"/>
       <c r="B91" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>82</v>
       </c>
       <c r="C91" s="58" t="s">
@@ -6717,16 +6781,17 @@
         <v>1</v>
       </c>
       <c r="L91" s="38">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M91" s="38">
         <v>100</v>
       </c>
-      <c r="M91" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N91" s="65">
+      <c r="N91" s="63">
         <v>0.1013</v>
       </c>
-      <c r="O91" s="65">
-        <f t="shared" si="2"/>
+      <c r="O91" s="63">
+        <f t="shared" si="4"/>
         <v>10.130000000000001</v>
       </c>
       <c r="P91" s="38"/>
@@ -6765,16 +6830,17 @@
         <v>5</v>
       </c>
       <c r="L92" s="36">
+        <f t="shared" si="5"/>
+        <v>50</v>
+      </c>
+      <c r="M92" s="36">
         <v>100</v>
       </c>
-      <c r="M92" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N92" s="63">
+      <c r="N92" s="62">
         <v>0.1014</v>
       </c>
-      <c r="O92" s="63">
-        <f t="shared" si="2"/>
+      <c r="O92" s="62">
+        <f t="shared" si="4"/>
         <v>10.14</v>
       </c>
       <c r="P92" s="36"/>
@@ -6782,7 +6848,7 @@
     <row r="93" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A93" s="1"/>
       <c r="B93" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>84</v>
       </c>
       <c r="C93" s="58" t="s">
@@ -6813,16 +6879,17 @@
         <v>2</v>
       </c>
       <c r="L93" s="38">
+        <f t="shared" si="5"/>
+        <v>20</v>
+      </c>
+      <c r="M93" s="38">
         <v>100</v>
       </c>
-      <c r="M93" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N93" s="65">
+      <c r="N93" s="63">
         <v>0.1014</v>
       </c>
-      <c r="O93" s="65">
-        <f t="shared" si="2"/>
+      <c r="O93" s="63">
+        <f t="shared" si="4"/>
         <v>10.14</v>
       </c>
       <c r="P93" s="38"/>
@@ -6861,16 +6928,17 @@
         <v>2</v>
       </c>
       <c r="L94" s="36">
+        <f t="shared" si="5"/>
+        <v>20</v>
+      </c>
+      <c r="M94" s="36">
         <v>100</v>
       </c>
-      <c r="M94" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N94" s="63">
+      <c r="N94" s="62">
         <v>0.10120000000000001</v>
       </c>
-      <c r="O94" s="63">
-        <f t="shared" si="2"/>
+      <c r="O94" s="62">
+        <f t="shared" si="4"/>
         <v>10.120000000000001</v>
       </c>
       <c r="P94" s="36"/>
@@ -6878,7 +6946,7 @@
     <row r="95" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A95" s="1"/>
       <c r="B95" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>86</v>
       </c>
       <c r="C95" s="58" t="s">
@@ -6909,16 +6977,17 @@
         <v>4</v>
       </c>
       <c r="L95" s="38">
+        <f t="shared" si="5"/>
+        <v>40</v>
+      </c>
+      <c r="M95" s="38">
         <v>45</v>
       </c>
-      <c r="M95" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N95" s="65">
+      <c r="N95" s="63">
         <v>0.1855</v>
       </c>
-      <c r="O95" s="65">
-        <f t="shared" si="2"/>
+      <c r="O95" s="63">
+        <f t="shared" si="4"/>
         <v>8.3475000000000001</v>
       </c>
       <c r="P95" s="38"/>
@@ -6957,16 +7026,17 @@
         <v>2</v>
       </c>
       <c r="L96" s="36">
+        <f t="shared" si="5"/>
+        <v>20</v>
+      </c>
+      <c r="M96" s="36">
         <v>50</v>
       </c>
-      <c r="M96" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N96" s="63">
+      <c r="N96" s="62">
         <v>0.10490000000000001</v>
       </c>
-      <c r="O96" s="63">
-        <f t="shared" si="2"/>
+      <c r="O96" s="62">
+        <f t="shared" si="4"/>
         <v>5.2450000000000001</v>
       </c>
       <c r="P96" s="36"/>
@@ -6974,7 +7044,7 @@
     <row r="97" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A97" s="1"/>
       <c r="B97" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>88</v>
       </c>
       <c r="C97" s="58" t="s">
@@ -7005,16 +7075,17 @@
         <v>2</v>
       </c>
       <c r="L97" s="38">
+        <f t="shared" si="5"/>
+        <v>20</v>
+      </c>
+      <c r="M97" s="38">
         <v>100</v>
       </c>
-      <c r="M97" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N97" s="65">
+      <c r="N97" s="63">
         <v>0.1014</v>
       </c>
-      <c r="O97" s="65">
-        <f t="shared" si="2"/>
+      <c r="O97" s="63">
+        <f t="shared" si="4"/>
         <v>10.14</v>
       </c>
       <c r="P97" s="38"/>
@@ -7053,16 +7124,17 @@
         <v>1</v>
       </c>
       <c r="L98" s="36">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M98" s="36">
         <v>20</v>
       </c>
-      <c r="M98" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N98" s="63">
+      <c r="N98" s="62">
         <v>0.1361</v>
       </c>
-      <c r="O98" s="63">
-        <f t="shared" si="2"/>
+      <c r="O98" s="62">
+        <f t="shared" si="4"/>
         <v>2.722</v>
       </c>
       <c r="P98" s="36"/>
@@ -7070,7 +7142,7 @@
     <row r="99" spans="1:16" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A99" s="1"/>
       <c r="B99" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>90</v>
       </c>
       <c r="C99" s="58" t="s">
@@ -7100,16 +7172,17 @@
       <c r="K99" s="39">
         <v>33</v>
       </c>
-      <c r="L99" s="38" t="s">
-        <v>480</v>
-      </c>
-      <c r="M99" s="64" t="s">
-        <v>480</v>
-      </c>
-      <c r="N99" s="65">
+      <c r="L99" s="38">
+        <f t="shared" si="5"/>
+        <v>330</v>
+      </c>
+      <c r="M99" s="38" t="s">
+        <v>480</v>
+      </c>
+      <c r="N99" s="63">
         <v>0</v>
       </c>
-      <c r="O99" s="65" t="s">
+      <c r="O99" s="63" t="s">
         <v>480</v>
       </c>
       <c r="P99" s="38"/>
@@ -7148,16 +7221,17 @@
         <v>7</v>
       </c>
       <c r="L100" s="36">
+        <f t="shared" si="5"/>
+        <v>70</v>
+      </c>
+      <c r="M100" s="36">
         <v>80</v>
       </c>
-      <c r="M100" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N100" s="63">
+      <c r="N100" s="62">
         <v>0.1595</v>
       </c>
-      <c r="O100" s="63">
-        <f t="shared" si="2"/>
+      <c r="O100" s="62">
+        <f t="shared" ref="O100:O119" si="6">N100*M100</f>
         <v>12.76</v>
       </c>
       <c r="P100" s="36"/>
@@ -7165,7 +7239,7 @@
     <row r="101" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A101" s="1"/>
       <c r="B101" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>92</v>
       </c>
       <c r="C101" s="58" t="s">
@@ -7174,41 +7248,42 @@
       <c r="D101" s="38" t="s">
         <v>97</v>
       </c>
-      <c r="E101" s="70" t="s">
+      <c r="E101" s="68" t="s">
         <v>208</v>
       </c>
-      <c r="F101" s="71" t="s">
+      <c r="F101" s="69" t="s">
         <v>487</v>
       </c>
-      <c r="G101" s="70" t="s">
+      <c r="G101" s="68" t="s">
         <v>266</v>
       </c>
-      <c r="H101" s="71" t="s">
-        <v>480</v>
-      </c>
-      <c r="I101" s="71" t="s">
+      <c r="H101" s="69" t="s">
+        <v>480</v>
+      </c>
+      <c r="I101" s="69" t="s">
         <v>393</v>
       </c>
-      <c r="J101" s="71" t="s">
-        <v>480</v>
-      </c>
-      <c r="K101" s="70">
+      <c r="J101" s="69" t="s">
+        <v>480</v>
+      </c>
+      <c r="K101" s="68">
         <v>1</v>
       </c>
-      <c r="L101" s="71">
+      <c r="L101" s="38">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M101" s="69">
         <v>11</v>
       </c>
-      <c r="M101" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N101" s="65">
+      <c r="N101" s="63">
         <v>0.3</v>
       </c>
-      <c r="O101" s="72">
-        <f t="shared" si="2"/>
+      <c r="O101" s="70">
+        <f t="shared" si="6"/>
         <v>3.3</v>
       </c>
-      <c r="P101" s="68"/>
+      <c r="P101" s="66"/>
     </row>
     <row r="102" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A102" s="1"/>
@@ -7244,16 +7319,17 @@
         <v>1</v>
       </c>
       <c r="L102" s="36">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M102" s="36">
         <v>12</v>
       </c>
-      <c r="M102" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N102" s="63">
+      <c r="N102" s="62">
         <v>0.66289999999999993</v>
       </c>
-      <c r="O102" s="63">
-        <f t="shared" si="2"/>
+      <c r="O102" s="62">
+        <f t="shared" si="6"/>
         <v>7.9547999999999988</v>
       </c>
       <c r="P102" s="36"/>
@@ -7261,7 +7337,7 @@
     <row r="103" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A103" s="1"/>
       <c r="B103" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>94</v>
       </c>
       <c r="C103" s="58" t="s">
@@ -7292,16 +7368,17 @@
         <v>2</v>
       </c>
       <c r="L103" s="38">
+        <f t="shared" si="5"/>
+        <v>20</v>
+      </c>
+      <c r="M103" s="38">
         <v>22</v>
       </c>
-      <c r="M103" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N103" s="65">
+      <c r="N103" s="63">
         <v>0.25480000000000003</v>
       </c>
-      <c r="O103" s="65">
-        <f t="shared" si="2"/>
+      <c r="O103" s="63">
+        <f t="shared" si="6"/>
         <v>5.6056000000000008</v>
       </c>
       <c r="P103" s="38"/>
@@ -7340,16 +7417,17 @@
         <v>1</v>
       </c>
       <c r="L104" s="36">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M104" s="36">
         <v>11</v>
       </c>
-      <c r="M104" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N104" s="63">
+      <c r="N104" s="62">
         <v>0.25559999999999999</v>
       </c>
-      <c r="O104" s="63">
-        <f t="shared" si="2"/>
+      <c r="O104" s="62">
+        <f t="shared" si="6"/>
         <v>2.8115999999999999</v>
       </c>
       <c r="P104" s="36"/>
@@ -7357,7 +7435,7 @@
     <row r="105" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A105" s="1"/>
       <c r="B105" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>96</v>
       </c>
       <c r="C105" s="58" t="s">
@@ -7388,16 +7466,17 @@
         <v>1</v>
       </c>
       <c r="L105" s="38">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M105" s="38">
         <v>12</v>
       </c>
-      <c r="M105" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N105" s="65">
+      <c r="N105" s="63">
         <v>0.29189999999999999</v>
       </c>
-      <c r="O105" s="65">
-        <f t="shared" si="2"/>
+      <c r="O105" s="63">
+        <f t="shared" si="6"/>
         <v>3.5027999999999997</v>
       </c>
       <c r="P105" s="38"/>
@@ -7436,16 +7515,17 @@
         <v>1</v>
       </c>
       <c r="L106" s="36">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M106" s="36">
         <v>15</v>
       </c>
-      <c r="M106" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N106" s="63">
+      <c r="N106" s="62">
         <v>0.23039999999999999</v>
       </c>
-      <c r="O106" s="63">
-        <f t="shared" si="2"/>
+      <c r="O106" s="62">
+        <f t="shared" si="6"/>
         <v>3.456</v>
       </c>
       <c r="P106" s="36"/>
@@ -7453,7 +7533,7 @@
     <row r="107" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A107" s="1"/>
       <c r="B107" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>98</v>
       </c>
       <c r="C107" s="58" t="s">
@@ -7484,16 +7564,17 @@
         <v>1</v>
       </c>
       <c r="L107" s="38">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M107" s="38">
         <v>12</v>
       </c>
-      <c r="M107" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N107" s="65">
+      <c r="N107" s="63">
         <v>0.41849999999999998</v>
       </c>
-      <c r="O107" s="65">
-        <f t="shared" si="2"/>
+      <c r="O107" s="63">
+        <f t="shared" si="6"/>
         <v>5.0220000000000002</v>
       </c>
       <c r="P107" s="38"/>
@@ -7532,16 +7613,17 @@
         <v>1</v>
       </c>
       <c r="L108" s="36">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M108" s="36">
         <v>11</v>
       </c>
-      <c r="M108" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N108" s="63">
+      <c r="N108" s="62">
         <v>2.06</v>
       </c>
-      <c r="O108" s="63">
-        <f t="shared" si="2"/>
+      <c r="O108" s="62">
+        <f t="shared" si="6"/>
         <v>22.66</v>
       </c>
       <c r="P108" s="36"/>
@@ -7549,7 +7631,7 @@
     <row r="109" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A109" s="1"/>
       <c r="B109" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>100</v>
       </c>
       <c r="C109" s="58" t="s">
@@ -7580,16 +7662,17 @@
         <v>1</v>
       </c>
       <c r="L109" s="38">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M109" s="38">
         <v>11</v>
       </c>
-      <c r="M109" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N109" s="65">
+      <c r="N109" s="63">
         <v>20.93</v>
       </c>
-      <c r="O109" s="65">
-        <f t="shared" si="2"/>
+      <c r="O109" s="63">
+        <f t="shared" si="6"/>
         <v>230.23</v>
       </c>
       <c r="P109" s="38"/>
@@ -7628,16 +7711,17 @@
         <v>2</v>
       </c>
       <c r="L110" s="36">
+        <f t="shared" si="5"/>
+        <v>20</v>
+      </c>
+      <c r="M110" s="36">
         <v>25</v>
       </c>
-      <c r="M110" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N110" s="63">
+      <c r="N110" s="62">
         <v>0.2409</v>
       </c>
-      <c r="O110" s="63">
-        <f t="shared" si="2"/>
+      <c r="O110" s="62">
+        <f t="shared" si="6"/>
         <v>6.0225</v>
       </c>
       <c r="P110" s="36"/>
@@ -7645,7 +7729,7 @@
     <row r="111" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A111" s="1"/>
       <c r="B111" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>102</v>
       </c>
       <c r="C111" s="58" t="s">
@@ -7676,16 +7760,17 @@
         <v>1</v>
       </c>
       <c r="L111" s="38">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M111" s="38">
         <v>11</v>
       </c>
-      <c r="M111" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N111" s="65">
+      <c r="N111" s="63">
         <v>0.96409999999999996</v>
       </c>
-      <c r="O111" s="65">
-        <f t="shared" si="2"/>
+      <c r="O111" s="63">
+        <f t="shared" si="6"/>
         <v>10.6051</v>
       </c>
       <c r="P111" s="38"/>
@@ -7724,16 +7809,17 @@
         <v>1</v>
       </c>
       <c r="L112" s="36">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M112" s="36">
         <v>11</v>
       </c>
-      <c r="M112" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N112" s="63">
+      <c r="N112" s="62">
         <v>6.3104999999999993</v>
       </c>
-      <c r="O112" s="63">
-        <f t="shared" si="2"/>
+      <c r="O112" s="62">
+        <f t="shared" si="6"/>
         <v>69.415499999999994</v>
       </c>
       <c r="P112" s="36"/>
@@ -7741,7 +7827,7 @@
     <row r="113" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A113" s="1"/>
       <c r="B113" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>104</v>
       </c>
       <c r="C113" s="58" t="s">
@@ -7772,16 +7858,17 @@
         <v>1</v>
       </c>
       <c r="L113" s="38">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M113" s="38">
         <v>11</v>
       </c>
-      <c r="M113" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N113" s="65">
+      <c r="N113" s="63">
         <v>14.936</v>
       </c>
-      <c r="O113" s="65">
-        <f t="shared" si="2"/>
+      <c r="O113" s="63">
+        <f t="shared" si="6"/>
         <v>164.29599999999999</v>
       </c>
       <c r="P113" s="38"/>
@@ -7820,16 +7907,17 @@
         <v>1</v>
       </c>
       <c r="L114" s="36">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M114" s="36">
         <v>11</v>
       </c>
-      <c r="M114" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N114" s="63">
+      <c r="N114" s="62">
         <v>13.7875</v>
       </c>
-      <c r="O114" s="63">
-        <f t="shared" si="2"/>
+      <c r="O114" s="62">
+        <f t="shared" si="6"/>
         <v>151.66249999999999</v>
       </c>
       <c r="P114" s="36"/>
@@ -7837,7 +7925,7 @@
     <row r="115" spans="1:16" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A115" s="1"/>
       <c r="B115" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>106</v>
       </c>
       <c r="C115" s="58" t="s">
@@ -7868,16 +7956,17 @@
         <v>1</v>
       </c>
       <c r="L115" s="38">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M115" s="38">
         <v>11</v>
       </c>
-      <c r="M115" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N115" s="65">
+      <c r="N115" s="63">
         <v>17.600000000000001</v>
       </c>
-      <c r="O115" s="65">
-        <f t="shared" si="2"/>
+      <c r="O115" s="63">
+        <f t="shared" si="6"/>
         <v>193.60000000000002</v>
       </c>
       <c r="P115" s="38"/>
@@ -7916,16 +8005,17 @@
         <v>2</v>
       </c>
       <c r="L116" s="36">
+        <f t="shared" si="5"/>
+        <v>20</v>
+      </c>
+      <c r="M116" s="36">
         <v>22</v>
       </c>
-      <c r="M116" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N116" s="63">
+      <c r="N116" s="62">
         <v>0.44950000000000001</v>
       </c>
-      <c r="O116" s="63">
-        <f t="shared" si="2"/>
+      <c r="O116" s="62">
+        <f t="shared" si="6"/>
         <v>9.8889999999999993</v>
       </c>
       <c r="P116" s="36"/>
@@ -7933,7 +8023,7 @@
     <row r="117" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A117" s="1"/>
       <c r="B117" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>108</v>
       </c>
       <c r="C117" s="58" t="s">
@@ -7964,16 +8054,17 @@
         <v>1</v>
       </c>
       <c r="L117" s="38">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M117" s="38">
         <v>15</v>
       </c>
-      <c r="M117" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N117" s="65">
+      <c r="N117" s="63">
         <v>0.1865</v>
       </c>
-      <c r="O117" s="65">
-        <f t="shared" si="2"/>
+      <c r="O117" s="63">
+        <f t="shared" si="6"/>
         <v>2.7974999999999999</v>
       </c>
       <c r="P117" s="38"/>
@@ -8012,16 +8103,17 @@
         <v>1</v>
       </c>
       <c r="L118" s="36">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M118" s="36">
         <v>11</v>
       </c>
-      <c r="M118" s="62" t="s">
-        <v>514</v>
-      </c>
-      <c r="N118" s="63">
+      <c r="N118" s="62">
         <v>0.26180000000000003</v>
       </c>
-      <c r="O118" s="63">
-        <f t="shared" si="2"/>
+      <c r="O118" s="62">
+        <f t="shared" si="6"/>
         <v>2.8798000000000004</v>
       </c>
       <c r="P118" s="36"/>
@@ -8029,7 +8121,7 @@
     <row r="119" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A119" s="1"/>
       <c r="B119" s="50">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>110</v>
       </c>
       <c r="C119" s="58" t="s">
@@ -8060,16 +8152,17 @@
         <v>1</v>
       </c>
       <c r="L119" s="38">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M119" s="38">
         <v>11</v>
       </c>
-      <c r="M119" s="64" t="s">
-        <v>514</v>
-      </c>
-      <c r="N119" s="65">
+      <c r="N119" s="63">
         <v>0.34360000000000002</v>
       </c>
-      <c r="O119" s="65">
-        <f t="shared" si="2"/>
+      <c r="O119" s="63">
+        <f t="shared" si="6"/>
         <v>3.7796000000000003</v>
       </c>
       <c r="P119" s="38"/>
@@ -8086,12 +8179,12 @@
       <c r="I120" s="34"/>
       <c r="J120" s="35"/>
       <c r="K120" s="35"/>
-      <c r="L120" s="76" t="s">
-        <v>510</v>
-      </c>
-      <c r="M120" s="77"/>
-      <c r="N120" s="77"/>
-      <c r="O120" s="66">
+      <c r="L120" s="35"/>
+      <c r="M120" s="74" t="s">
+        <v>509</v>
+      </c>
+      <c r="N120" s="75"/>
+      <c r="O120" s="64">
         <f>SUM(O10:O119)</f>
         <v>1787.6428999999998</v>
       </c>
@@ -8109,12 +8202,12 @@
       <c r="I121" s="9"/>
       <c r="J121" s="9"/>
       <c r="K121" s="9"/>
-      <c r="L121" s="76" t="s">
-        <v>511</v>
-      </c>
-      <c r="M121" s="77"/>
-      <c r="N121" s="77"/>
-      <c r="O121" s="67">
+      <c r="L121" s="9"/>
+      <c r="M121" s="74" t="s">
+        <v>510</v>
+      </c>
+      <c r="N121" s="75"/>
+      <c r="O121" s="65">
         <f>O120/10</f>
         <v>178.76428999999999</v>
       </c>
@@ -8124,8 +8217,8 @@
   <mergeCells count="4">
     <mergeCell ref="J1:P1"/>
     <mergeCell ref="P3:P8"/>
-    <mergeCell ref="L120:N120"/>
-    <mergeCell ref="L121:N121"/>
+    <mergeCell ref="M120:N120"/>
+    <mergeCell ref="M121:N121"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>